<commit_message>
fix(vilextime): rewrite or replace every khong_dat row
56 lineages get a rewritten question (validate() as before, model question
kept in model_question, edited_by claude-opus-5-5) and their model labels
re-judged in place. 19 unfixable lineages, plus one T3 lineage with only two
distinct answers, go to data/vilextime/dropped.jsonl; --select skips them so
the next ranked lineages fill the quota (7 reserve, 12 new questions).
audit-sheet reads dropped rows from their group file and shows the drop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/audit_T4.xlsx
+++ b/data/review/audit_T4.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R38"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,15 +494,20 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>audit</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>auditor</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>audit_note</t>
         </is>
@@ -521,7 +526,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Trường hợp quận, thành phố thuộc thành phố trực thuộc trung ương đã có quy hoạch được phê duyệt, loại quy hoạch nào cho phép không phải lập quy hoạch sử dụng đất cấp huyện?</t>
+          <t>Quy hoạch chung hoặc quy hoạch phân khu cho phép quận, thành phố thuộc thành phố trực thuộc trung ương không phải lập quy hoạch sử dụng đất cấp huyện phải được phê duyệt theo pháp luật về lĩnh vực nào?</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -561,24 +566,21 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Loại quy hoạch (quy hoạch chung hoặc quy hoạch phân khu) như nhau ở hai mốc; chỉ đổi tên luật dẫn chiếu (quy hoạch đô thị → quy hoạch đô thị và nông thôn)</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp quận, thành phố thuộc thành phố trực thuộc trung ương đã có quy hoạch được phê duyệt, loại quy hoạch nào cho phép không phải lập quy hoạch sử dụng đất cấp huyện?»; nhãn cũ khong_dat group_mismatch: Loại quy hoạch (quy hoạch chung hoặc quy hoạch phân khu) như nhau ở hai mốc; chỉ đổi tên luật dẫn chiếu (quy hoạch đô thị → quy hoạch đô thị và nông thôn)). Câu hỏi hỏi pháp luật phê duyệt, chạm chỗ đổi tên luật</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -593,7 +595,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Trường hợp quận, thành phố thuộc thành phố trực thuộc trung ương đã có quy hoạch được phê duyệt, loại quy hoạch nào cho phép không phải lập quy hoạch sử dụng đất cấp huyện?</t>
+          <t>Quy hoạch chung hoặc quy hoạch phân khu cho phép quận, thành phố thuộc thành phố trực thuộc trung ương không phải lập quy hoạch sử dụng đất cấp huyện phải được phê duyệt theo pháp luật về lĩnh vực nào?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -633,24 +635,21 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Loại quy hoạch (quy hoạch chung hoặc quy hoạch phân khu) như nhau ở hai mốc; chỉ đổi tên luật dẫn chiếu (quy hoạch đô thị → quy hoạch đô thị và nông thôn)</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp quận, thành phố thuộc thành phố trực thuộc trung ương đã có quy hoạch được phê duyệt, loại quy hoạch nào cho phép không phải lập quy hoạch sử dụng đất cấp huyện?»; nhãn cũ khong_dat group_mismatch: Loại quy hoạch (quy hoạch chung hoặc quy hoạch phân khu) như nhau ở hai mốc; chỉ đổi tên luật dẫn chiếu (quy hoạch đô thị → quy hoạch đô thị và nông thôn)). Câu hỏi hỏi pháp luật phê duyệt, chạm chỗ đổi tên luật</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -724,9 +723,14 @@
           <t>b) Nhân viên của doanh nghiệp giao nhận hàng hóa, bưu gửi bằng đường hàng không;</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>loại lineage (question_ambiguous): Điểm b (doanh nghiệp giao nhận hàng hóa, bưu gửi bằng đường hàng không) và điểm c (doanh nghiệp khảo sát, thi công, sửa chữa, bảo dưỡng tại cảng) cùng khoản cũng là doanh nghiệp có nhân viên được xem xét cấp thẻ dài hạn</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -800,9 +804,14 @@
           <t>b) Nhân viên của doanh nghiệp giao nhận hàng hóa, bưu gửi bằng đường hàng không;</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>loại lineage (question_ambiguous): Điểm b (doanh nghiệp giao nhận hàng hóa, bưu gửi bằng đường hàng không) và điểm c (doanh nghiệp khảo sát, thi công, sửa chữa, bảo dưỡng tại cảng) cùng khoản cũng là doanh nghiệp có nhân viên được xem xét cấp thẻ dài hạn</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -871,6 +880,7 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -935,6 +945,7 @@
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -999,6 +1010,7 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1063,6 +1075,7 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1077,7 +1090,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Theo quy định về di dời trạm định vị vệ tinh, Ủy ban nhân dân cấp tỉnh phối hợp với bộ nào để thực hiện?</t>
+          <t>Khi di dời trạm định vị vệ tinh quốc gia, Ủy ban nhân dân cấp tỉnh phối hợp với bộ nào để tổ chức việc di dời?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1117,28 +1130,21 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Câu hỏi không nêu trạm quốc gia; điểm đ cùng khoản quy định Ủy ban nhân dân cấp tỉnh phối hợp với bộ, cơ quan ngang bộ, cơ quan thuộc Chính phủ di dời trạm định vị vệ tinh chuyên ngành</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>đ) Ủy ban nhân dân cấp tỉnh phối hợp với bộ, cơ quan ngang bộ, cơ quan thuộc Chính phủ tổ chức việc di dời trạ...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Theo quy định về di dời trạm định vị vệ tinh, Ủy ban nhân dân cấp tỉnh phối hợp với bộ nào để thực hiện?»; nhãn cũ khong_dat question_ambiguous: Câu hỏi không nêu trạm quốc gia; điểm đ cùng khoản quy định Ủy ban nhân dân cấp tỉnh phối hợp với bộ, cơ quan ngang bộ, cơ quan thuộc Chính phủ di dời trạm định vị vệ tinh chuyên ngành). Đã nêu trạm quốc gia, loại điểm đ</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1153,7 +1159,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Theo quy định về di dời trạm định vị vệ tinh, Ủy ban nhân dân cấp tỉnh phối hợp với bộ nào để thực hiện?</t>
+          <t>Khi di dời trạm định vị vệ tinh quốc gia, Ủy ban nhân dân cấp tỉnh phối hợp với bộ nào để tổ chức việc di dời?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1193,28 +1199,21 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Câu hỏi không nêu trạm quốc gia; điểm đ cùng khoản quy định Ủy ban nhân dân cấp tỉnh phối hợp với bộ, cơ quan ngang bộ, cơ quan thuộc Chính phủ di dời trạm định vị vệ tinh chuyên ngành</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>đ) Ủy ban nhân dân cấp tỉnh phối hợp với bộ, cơ quan ngang bộ, cơ quan thuộc Chính phủ tổ chức việc di dời trạ...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Theo quy định về di dời trạm định vị vệ tinh, Ủy ban nhân dân cấp tỉnh phối hợp với bộ nào để thực hiện?»; nhãn cũ khong_dat question_ambiguous: Câu hỏi không nêu trạm quốc gia; điểm đ cùng khoản quy định Ủy ban nhân dân cấp tỉnh phối hợp với bộ, cơ quan ngang bộ, cơ quan thuộc Chính phủ di dời trạm định vị vệ tinh chuyên ngành). Đã nêu trạm quốc gia, loại điểm đ</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1229,7 +1228,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Khi sĩ quan dự bị vắng mặt tại nơi cư trú từ 30 ngày trở lên, người đó phải báo cáo cho cơ quan quân sự cấp nào và theo thời gian nào?</t>
+          <t>Khi có sĩ quan dự bị vắng mặt tại nơi cư trú, Ban Chỉ huy quân sự cấp xã phải tổng hợp báo cáo lên cơ quan quân sự nào và vào thời gian nào?</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1269,24 +1268,21 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Người vắng mặt báo cáo Ban Chỉ huy quân sự cấp xã (hoặc nơi làm việc) ở cả hai mốc; chỗ đổi là việc Ban Chỉ huy quân sự cấp xã tổng hợp báo cáo lên cấp huyện → cấp tỉnh, từ ngày 25 đến 30 hằng tháng</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi sĩ quan dự bị vắng mặt tại nơi cư trú từ 30 ngày trở lên, người đó phải báo cáo cho cơ quan quân sự cấp nào và theo thời gian nào?»; nhãn cũ khong_dat group_mismatch: Người vắng mặt báo cáo Ban Chỉ huy quân sự cấp xã (hoặc nơi làm việc) ở cả hai mốc; chỗ đổi là việc Ban Chỉ huy quân sự cấp xã tổng hợp báo cáo lên cấp huyện → cấp tỉnh, từ ngày 25 đến 30 hằng tháng). Câu hỏi hỏi nơi nhận và thời gian báo cáo tổng hợp, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1301,7 +1297,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Khi sĩ quan dự bị vắng mặt tại nơi cư trú từ 30 ngày trở lên, người đó phải báo cáo cho cơ quan quân sự cấp nào và theo thời gian nào?</t>
+          <t>Khi có sĩ quan dự bị vắng mặt tại nơi cư trú, Ban Chỉ huy quân sự cấp xã phải tổng hợp báo cáo lên cơ quan quân sự nào và vào thời gian nào?</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1341,24 +1337,21 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Người vắng mặt báo cáo Ban Chỉ huy quân sự cấp xã (hoặc nơi làm việc) ở cả hai mốc; chỗ đổi là việc Ban Chỉ huy quân sự cấp xã tổng hợp báo cáo lên cấp huyện → cấp tỉnh, từ ngày 25 đến 30 hằng tháng</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi sĩ quan dự bị vắng mặt tại nơi cư trú từ 30 ngày trở lên, người đó phải báo cáo cho cơ quan quân sự cấp nào và theo thời gian nào?»; nhãn cũ khong_dat group_mismatch: Người vắng mặt báo cáo Ban Chỉ huy quân sự cấp xã (hoặc nơi làm việc) ở cả hai mốc; chỗ đổi là việc Ban Chỉ huy quân sự cấp xã tổng hợp báo cáo lên cấp huyện → cấp tỉnh, từ ngày 25 đến 30 hằng tháng). Câu hỏi hỏi nơi nhận và thời gian báo cáo tổng hợp, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1423,6 +1416,7 @@
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1487,6 +1481,7 @@
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1551,6 +1546,7 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1615,6 +1611,7 @@
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1629,7 +1626,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Trường hợp cấp Giấy chứng nhận vùng hoạt động hoa tiêu hàng hải cho một vùng và tuyến dẫn tàu cụ thể, người được cấp phải đáp ứng điều kiện gì về thực tập dẫn tàu?</t>
+          <t>Những người nào được cấp Giấy chứng nhận vùng hoạt động hoa tiêu hàng hải tại một vùng hoạt động và tuyến dẫn tàu căn cứ vào kinh nghiệm đã có tại vùng, tuyến đó?</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1669,24 +1666,21 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Với hoa tiêu, điều kiện thực tập dẫn tàu như nhau ở hai mốc; chỗ đổi thêm trường hợp thuyền trưởng đã dẫn tàu, câu hỏi không hỏi</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp cấp Giấy chứng nhận vùng hoạt động hoa tiêu hàng hải cho một vùng và tuyến dẫn tàu cụ thể, người được cấp phải đáp ứng điều kiện gì về thực tập dẫn tàu?»; nhãn cũ khong_dat group_mismatch: Với hoa tiêu, điều kiện thực tập dẫn tàu như nhau ở hai mốc; chỗ đổi thêm trường hợp thuyền trưởng đã dẫn tàu, câu hỏi không hỏi). Câu hỏi hỏi những người được cấp theo kinh nghiệm, chạm chỗ thêm thuyền trưởng</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1701,7 +1695,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Trường hợp cấp Giấy chứng nhận vùng hoạt động hoa tiêu hàng hải cho một vùng và tuyến dẫn tàu cụ thể, người được cấp phải đáp ứng điều kiện gì về thực tập dẫn tàu?</t>
+          <t>Những người nào được cấp Giấy chứng nhận vùng hoạt động hoa tiêu hàng hải tại một vùng hoạt động và tuyến dẫn tàu căn cứ vào kinh nghiệm đã có tại vùng, tuyến đó?</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1741,24 +1735,21 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Với hoa tiêu, điều kiện thực tập dẫn tàu như nhau ở hai mốc; chỗ đổi thêm trường hợp thuyền trưởng đã dẫn tàu, câu hỏi không hỏi</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp cấp Giấy chứng nhận vùng hoạt động hoa tiêu hàng hải cho một vùng và tuyến dẫn tàu cụ thể, người được cấp phải đáp ứng điều kiện gì về thực tập dẫn tàu?»; nhãn cũ khong_dat group_mismatch: Với hoa tiêu, điều kiện thực tập dẫn tàu như nhau ở hai mốc; chỗ đổi thêm trường hợp thuyền trưởng đã dẫn tàu, câu hỏi không hỏi). Câu hỏi hỏi những người được cấp theo kinh nghiệm, chạm chỗ thêm thuyền trưởng</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1773,7 +1764,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Một người lao động Việt Nam đăng ký dự tuyển làm việc cho tổ chức nước ngoài thì văn bằng, chứng chỉ trong hồ sơ được nộp dưới hình thức bản sao nào?</t>
+          <t>Văn bằng, chứng chỉ do nước ngoài cấp trong hồ sơ dự tuyển của người lao động Việt Nam làm việc cho tổ chức nước ngoài phải được dịch ra tiếng Việt và xác nhận bản dịch theo hình thức nào?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1813,24 +1804,21 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Câu hỏi hỏi hình thức bản sao: cả hai mốc đều là bản sao có chứng thực; chỗ đổi là bản dịch văn bằng nước ngoài được công chứng hoặc chứng thực, câu hỏi không hỏi</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Một người lao động Việt Nam đăng ký dự tuyển làm việc cho tổ chức nước ngoài thì văn bằng, chứng chỉ trong hồ sơ được nộp dưới hình thức bản sao nào?»; nhãn cũ khong_dat group_mismatch: Câu hỏi hỏi hình thức bản sao: cả hai mốc đều là bản sao có chứng thực; chỗ đổi là bản dịch văn bằng nước ngoài được công chứng hoặc chứng thực, câu hỏi không hỏi). Câu hỏi hỏi hình thức xác nhận bản dịch, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1845,7 +1833,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Một người lao động Việt Nam đăng ký dự tuyển làm việc cho tổ chức nước ngoài thì văn bằng, chứng chỉ trong hồ sơ được nộp dưới hình thức bản sao nào?</t>
+          <t>Văn bằng, chứng chỉ do nước ngoài cấp trong hồ sơ dự tuyển của người lao động Việt Nam làm việc cho tổ chức nước ngoài phải được dịch ra tiếng Việt và xác nhận bản dịch theo hình thức nào?</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1885,24 +1873,21 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Câu hỏi hỏi hình thức bản sao: cả hai mốc đều là bản sao có chứng thực; chỗ đổi là bản dịch văn bằng nước ngoài được công chứng hoặc chứng thực, câu hỏi không hỏi</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Một người lao động Việt Nam đăng ký dự tuyển làm việc cho tổ chức nước ngoài thì văn bằng, chứng chỉ trong hồ sơ được nộp dưới hình thức bản sao nào?»; nhãn cũ khong_dat group_mismatch: Câu hỏi hỏi hình thức bản sao: cả hai mốc đều là bản sao có chứng thực; chỗ đổi là bản dịch văn bằng nước ngoài được công chứng hoặc chứng thực, câu hỏi không hỏi). Câu hỏi hỏi hình thức xác nhận bản dịch, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1917,7 +1902,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Khi văn bản thông báo kết quả xác định trước mã số, xuất xứ, trị giá hải quan cần được xem xét lại, cơ quan hải quan cấp nào có thẩm quyền đối với văn bản này?</t>
+          <t>Trường hợp tổ chức, cá nhân không đồng ý với kết quả xác định trước mã số, xuất xứ, trị giá hải quan nhưng cần thông quan hàng hóa, kết quả đó do người đứng đầu cơ quan hải quan cấp nào đưa ra và họ phải làm gì để được thông quan?</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1957,28 +1942,21 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Việc đề nghị xem xét lại văn bản xác định trước là nội dung khoản 5 cùng Điều; khoản 4 chỉ nói văn bản là cơ sở khai hải quan và cách thông quan khi không đồng ý. Câu hỏi 'cơ quan cấp nào có thẩm quyền đối với văn bản cần xem xét lại' khớp khoản 5 hơn</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>5. Trường hợp không đồng ý với nội dung xác định trước mã số, xuất xứ, trị giá hải quan, tổ chức, cá nhân có v...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi văn bản thông báo kết quả xác định trước mã số, xuất xứ, trị giá hải quan cần được xem xét lại, cơ quan hải quan cấp nào có thẩm quyền đối với văn bản này?»; nhãn cũ khong_dat question_ambiguous: Việc đề nghị xem xét lại văn bản xác định trước là nội dung khoản 5 cùng Điều; khoản 4 chỉ nói văn bản là cơ sở khai hải quan và cách thông quan khi không đồng ý. Câu hỏi 'cơ quan cấp nào có thẩm quyền đối với văn bản cần xem xét lại' khớp khoản 5 hơn). Câu hỏi không còn hỏi việc xem xét lại (khoản 5); hỏi người ra kết quả và cách thông quan</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1993,7 +1971,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Khi văn bản thông báo kết quả xác định trước mã số, xuất xứ, trị giá hải quan cần được xem xét lại, cơ quan hải quan cấp nào có thẩm quyền đối với văn bản này?</t>
+          <t>Trường hợp tổ chức, cá nhân không đồng ý với kết quả xác định trước mã số, xuất xứ, trị giá hải quan nhưng cần thông quan hàng hóa, kết quả đó do người đứng đầu cơ quan hải quan cấp nào đưa ra và họ phải làm gì để được thông quan?</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2033,28 +2011,21 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Việc đề nghị xem xét lại văn bản xác định trước là nội dung khoản 5 cùng Điều; khoản 4 chỉ nói văn bản là cơ sở khai hải quan và cách thông quan khi không đồng ý. Câu hỏi 'cơ quan cấp nào có thẩm quyền đối với văn bản cần xem xét lại' khớp khoản 5 hơn</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>5. Trường hợp không đồng ý với nội dung xác định trước mã số, xuất xứ, trị giá hải quan, tổ chức, cá nhân có v...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi văn bản thông báo kết quả xác định trước mã số, xuất xứ, trị giá hải quan cần được xem xét lại, cơ quan hải quan cấp nào có thẩm quyền đối với văn bản này?»; nhãn cũ khong_dat question_ambiguous: Việc đề nghị xem xét lại văn bản xác định trước là nội dung khoản 5 cùng Điều; khoản 4 chỉ nói văn bản là cơ sở khai hải quan và cách thông quan khi không đồng ý. Câu hỏi 'cơ quan cấp nào có thẩm quyền đối với văn bản cần xem xét lại' khớp khoản 5 hơn). Câu hỏi không còn hỏi việc xem xét lại (khoản 5); hỏi người ra kết quả và cách thông quan</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2069,7 +2040,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Trường hợp một tổ chức được chỉ định kiểm định phương tiện đo, quyết định chỉ định được gửi tới những cơ quan nào?</t>
+          <t>Sau khi ban hành, quyết định chỉ định tổ chức kiểm định phương tiện đo được gửi tới đâu và được đăng tải trên cổng thông tin điện tử của cơ quan nào?</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2109,24 +2080,21 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Nơi nhận quyết định (tổ chức được chỉ định, Chi cục Tiêu chuẩn Đo lường Chất lượng) như nhau ở hai mốc; chỗ đổi chỉ là cổng thông tin đăng tải (Tổng cục → Ủy ban), câu hỏi không hỏi tới</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp một tổ chức được chỉ định kiểm định phương tiện đo, quyết định chỉ định được gửi tới những cơ quan nào?»; nhãn cũ khong_dat group_mismatch: Nơi nhận quyết định (tổ chức được chỉ định, Chi cục Tiêu chuẩn Đo lường Chất lượng) như nhau ở hai mốc; chỗ đổi chỉ là cổng thông tin đăng tải (Tổng cục → Ủy ban), câu hỏi không hỏi tới). Câu hỏi nay hỏi cả cổng đăng tải, chạm chỗ đổi Tổng cục → Ủy ban</t>
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2141,7 +2109,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Trường hợp một tổ chức được chỉ định kiểm định phương tiện đo, quyết định chỉ định được gửi tới những cơ quan nào?</t>
+          <t>Sau khi ban hành, quyết định chỉ định tổ chức kiểm định phương tiện đo được gửi tới đâu và được đăng tải trên cổng thông tin điện tử của cơ quan nào?</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2181,24 +2149,21 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Nơi nhận quyết định (tổ chức được chỉ định, Chi cục Tiêu chuẩn Đo lường Chất lượng) như nhau ở hai mốc; chỗ đổi chỉ là cổng thông tin đăng tải (Tổng cục → Ủy ban), câu hỏi không hỏi tới</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp một tổ chức được chỉ định kiểm định phương tiện đo, quyết định chỉ định được gửi tới những cơ quan nào?»; nhãn cũ khong_dat group_mismatch: Nơi nhận quyết định (tổ chức được chỉ định, Chi cục Tiêu chuẩn Đo lường Chất lượng) như nhau ở hai mốc; chỗ đổi chỉ là cổng thông tin đăng tải (Tổng cục → Ủy ban), câu hỏi không hỏi tới). Câu hỏi nay hỏi cả cổng đăng tải, chạm chỗ đổi Tổng cục → Ủy ban</t>
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2213,7 +2178,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Khi Chấp hành viên gửi báo cáo thống kê kết quả thi hành án của kỳ trước, thời hạn chậm nhất là trước ngày nào của kỳ báo cáo kế tiếp?</t>
+          <t>Khi Chấp hành viên của cơ quan thi hành án dân sự không thuộc quân đội gửi báo cáo thống kê kết quả thi hành án của kỳ trước cho Thủ trưởng cơ quan nơi công tác, thời hạn chậm nhất là trước ngày nào của kỳ báo cáo kế tiếp?</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2253,28 +2218,21 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Câu hỏi không phân biệt Chấp hành viên dân sự (điểm a) với Chấp hành viên thi hành án dân sự trong quân đội (điểm d, vẫn trước ngày 03); ở mốc 2 hai điểm cho hai đáp án khác nhau</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>d) Chậm nhất trước ngày 03 của kỳ báo cáo kế tiếp, Chấp hành viên thi hành án dân sự trong quân đội phải gửi b...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi Chấp hành viên gửi báo cáo thống kê kết quả thi hành án của kỳ trước, thời hạn chậm nhất là trước ngày nào của kỳ báo cáo kế tiếp?»; nhãn cũ khong_dat question_ambiguous: Câu hỏi không phân biệt Chấp hành viên dân sự (điểm a) với Chấp hành viên thi hành án dân sự trong quân đội (điểm d, vẫn trước ngày 03); ở mốc 2 hai điểm cho hai đáp án khác nhau). Câu hỏi loại Chấp hành viên trong quân đội (điểm d)</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2289,7 +2247,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Khi Chấp hành viên gửi báo cáo thống kê kết quả thi hành án của kỳ trước, thời hạn chậm nhất là trước ngày nào của kỳ báo cáo kế tiếp?</t>
+          <t>Khi Chấp hành viên của cơ quan thi hành án dân sự không thuộc quân đội gửi báo cáo thống kê kết quả thi hành án của kỳ trước cho Thủ trưởng cơ quan nơi công tác, thời hạn chậm nhất là trước ngày nào của kỳ báo cáo kế tiếp?</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2329,28 +2287,21 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Câu hỏi không phân biệt Chấp hành viên dân sự (điểm a) với Chấp hành viên thi hành án dân sự trong quân đội (điểm d, vẫn trước ngày 03); ở mốc 2 hai điểm cho hai đáp án khác nhau</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>d) Chậm nhất trước ngày 03 của kỳ báo cáo kế tiếp, Chấp hành viên thi hành án dân sự trong quân đội phải gửi b...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi Chấp hành viên gửi báo cáo thống kê kết quả thi hành án của kỳ trước, thời hạn chậm nhất là trước ngày nào của kỳ báo cáo kế tiếp?»; nhãn cũ khong_dat question_ambiguous: Câu hỏi không phân biệt Chấp hành viên dân sự (điểm a) với Chấp hành viên thi hành án dân sự trong quân đội (điểm d, vẫn trước ngày 03); ở mốc 2 hai điểm cho hai đáp án khác nhau). Câu hỏi loại Chấp hành viên trong quân đội (điểm d)</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2365,7 +2316,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Trường hợp đầu tư nâng cao năng lực cho Cảnh sát môi trường, lực lượng này được đầu tư những gì và để đáp ứng yêu cầu công tác nào?</t>
+          <t>Theo quy định về đầu tư nâng cao năng lực, lực lượng cảnh sát nào được đầu tư cơ sở vật chất, phương tiện, thiết bị kỹ thuật để đấu tranh với tội phạm, vi phạm trong lĩnh vực môi trường?</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2405,24 +2356,21 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Nội dung đầu tư và yêu cầu công tác như nhau ở hai mốc; chỉ đổi tên lực lượng</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp đầu tư nâng cao năng lực cho Cảnh sát môi trường, lực lượng này được đầu tư những gì và để đáp ứng yêu cầu công tác nào?»; nhãn cũ khong_dat group_mismatch: Nội dung đầu tư và yêu cầu công tác như nhau ở hai mốc; chỉ đổi tên lực lượng). Câu hỏi hỏi tên lực lượng, không chép tên</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2437,7 +2385,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Trường hợp đầu tư nâng cao năng lực cho Cảnh sát môi trường, lực lượng này được đầu tư những gì và để đáp ứng yêu cầu công tác nào?</t>
+          <t>Theo quy định về đầu tư nâng cao năng lực, lực lượng cảnh sát nào được đầu tư cơ sở vật chất, phương tiện, thiết bị kỹ thuật để đấu tranh với tội phạm, vi phạm trong lĩnh vực môi trường?</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2477,29 +2425,26 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Nội dung đầu tư và yêu cầu công tác như nhau ở hai mốc; chỉ đổi tên lực lượng</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Trường hợp đầu tư nâng cao năng lực cho Cảnh sát môi trường, lực lượng này được đầu tư những gì và để đáp ứng yêu cầu công tác nào?»; nhãn cũ khong_dat group_mismatch: Nội dung đầu tư và yêu cầu công tác như nhau ở hai mốc; chỉ đổi tên lực lượng). Câu hỏi hỏi tên lực lượng, không chép tên</t>
         </is>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:a324f2cc-df4c-11f0-894a-8ddf853d159d:2024-01-31</t>
+          <t>vilextime:T4:provision:9d44166a-2e81-11f1-8975-ef6a7728f53c:2025-07-20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2509,37 +2454,37 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Trong lĩnh vực quản lý rừng bền vững, Sở Nông nghiệp và Phát triển nông thôn phải báo cáo kết quả hằng năm trước ngày nào và gửi cho đơn vị nào thuộc Bộ?</t>
+          <t>Trường hợp cần hướng dẫn thực hiện chế độ cho đối tượng mới được bổ sung, những bộ nào phải ban hành thông tư liên tịch?</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2025-07-20</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>3. Sở Nông nghiệp và Phát triển nông thôn:</t>
+          <t>Điều 3. Trách nhiệm thi hành</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>c) Hằng năm trước ngày 15 tháng 12, báo cáo Ủy ban nhân dân cấp tỉnh và Bộ Nông nghiệp và Phát triển nông thôn (Tổng cục Lâm nghiệp) kết quả xây dựng và thực hiện phương án quản lý rừng bền vững và cấp chứng chỉ quản lý rừng bền vững trên địa bàn tỉnh.</t>
+          <t>2. Bộ Công an, Bộ Lao động - Thương binh và Xã hội, Bộ Tài chính ban hành Thông tư liên tịch hướng dẫn thực hiện chế độ đối với đối tượng quy định tại khoản 3 Điều 1 Nghị định này.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Điểm c Khoản 3 Điều 18</t>
+          <t>Khoản 2 Điều 3</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>28/2018/TT-BNNPTNT</t>
+          <t>11/2011/NĐ-CP</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133923</t>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=26088</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2559,11 +2504,12 @@
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:ada68200-2d45-11f1-95b6-e35525714d94:2024-11-21</t>
+          <t>vilextime:T4:provision:a324f2cc-df4c-11f0-894a-8ddf853d159d:2024-01-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2573,37 +2519,37 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pháp luật về xây dựng và áp dụng tiêu chuẩn quy định cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch 5 năm xây dựng TCVN?</t>
+          <t>Trong lĩnh vực quản lý rừng bền vững, Sở Nông nghiệp và Phát triển nông thôn phải báo cáo kết quả hằng năm trước ngày nào và gửi cho đơn vị nào thuộc Bộ?</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2024-11-21</t>
+          <t>2024-01-31</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2. Kế hoạch 5 năm xây dựng TCVN Nội dung kế hoạch 5 năm xây dựng TCVN bao gồm: lĩnh vực, đối tượng cụ thể cần xây dựng TCVN; loại tiêu chuẩn; số lượng TCVN cần xây dựng; thời gian thực hiện; nguồn kinh phí và kinh phí dự kiến. Lập, phê duyệt, điều chỉnh, bổ sung kế hoạch 5 năm xây dựng TCVN thực hiện theo trình tự sau đây:</t>
+          <t>3. Sở Nông nghiệp và Phát triển nông thôn:</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>c) Phê duyệt kế hoạch 5 năm Bộ trưởng Bộ Khoa học và Công nghệ tổ chức xem xét, phê duyệt kế hoạch 5 năm xây dựng TCVN. Bộ Khoa học và Công nghệ thông báo kế hoạch đã được phê duyệt đến các bộ, ngành, tổ chức liên quan và công khai trên Cổng thông tin điện tử của Bộ Khoa học và Công nghệ, Cổng thông tin điện tử của Tổng cục Tiêu chuẩn Đo lường Chất lượng trong thời hạn 30 (ba mươi) ngày, kể từ ngày kế hoạch được phê duyệt;</t>
+          <t>c) Hằng năm trước ngày 15 tháng 12, báo cáo Ủy ban nhân dân cấp tỉnh và Bộ Nông nghiệp và Phát triển nông thôn (Tổng cục Lâm nghiệp) kết quả xây dựng và thực hiện phương án quản lý rừng bền vững và cấp chứng chỉ quản lý rừng bền vững trên địa bàn tỉnh.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Điểm c Khoản 2 Điều 4</t>
+          <t>Điểm c Khoản 3 Điều 18</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>11/2021/TT-BKHCN</t>
+          <t>28/2018/TT-BNNPTNT</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152575</t>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=133923</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2613,33 +2559,22 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>'Cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch' không ghim được chỗ đổi (cổng thông tin công khai); điểm b cùng khoản giao Tổng cục lấy ý kiến, hoàn chỉnh dự thảo kế hoạch, và điểm c do Bộ trưởng phê duyệt, Bộ thông báo</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>b) Lấy ý kiến và hoàn chỉnh dự thảo kế hoạch 5 năm Tổng cục Tiêu chuẩn Đo lường Chất lượng thực hiện các nhiệm...</t>
-        </is>
-      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:ada68200-2d45-11f1-95b6-e35525714d94:2024-11-22</t>
+          <t>vilextime:T4:provision:ada68200-2d45-11f1-95b6-e35525714d94:2024-11-21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2649,12 +2584,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pháp luật về xây dựng và áp dụng tiêu chuẩn quy định cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch 5 năm xây dựng TCVN?</t>
+          <t>Sau khi kế hoạch 5 năm xây dựng TCVN được phê duyệt, kế hoạch phải được công khai trên cổng thông tin điện tử của những cơ quan nào và trong thời hạn bao lâu?</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2024-11-22</t>
+          <t>2024-11-21</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2664,7 +2599,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>c) Phê duyệt kế hoạch 5 năm Bộ trưởng Bộ Khoa học và Công nghệ tổ chức xem xét, phê duyệt kế hoạch 5 năm xây dựng TCVN. Bộ Khoa học và Công nghệ thông báo kế hoạch đã được phê duyệt đến các bộ, ngành, tổ chức liên quan và công khai trên Cổng thông tin điện tử của Bộ Khoa học và Công nghệ, Cổng thông tin điện tử của Ủy ban Tiêu chuẩn Đo lường Chất lượng Quốc gia trong thời hạn 30 (ba mươi) ngày, kể từ ngày kế hoạch được phê duyệt;</t>
+          <t>c) Phê duyệt kế hoạch 5 năm Bộ trưởng Bộ Khoa học và Công nghệ tổ chức xem xét, phê duyệt kế hoạch 5 năm xây dựng TCVN. Bộ Khoa học và Công nghệ thông báo kế hoạch đã được phê duyệt đến các bộ, ngành, tổ chức liên quan và công khai trên Cổng thông tin điện tử của Bộ Khoa học và Công nghệ, Cổng thông tin điện tử của Tổng cục Tiêu chuẩn Đo lường Chất lượng trong thời hạn 30 (ba mươi) ngày, kể từ ngày kế hoạch được phê duyệt;</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2689,33 +2624,26 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>question_ambiguous</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
-          <t>'Cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch' không ghim được chỗ đổi (cổng thông tin công khai); điểm b cùng khoản giao Tổng cục lấy ý kiến, hoàn chỉnh dự thảo kế hoạch, và điểm c do Bộ trưởng phê duyệt, Bộ thông báo</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>b) Lấy ý kiến và hoàn chỉnh dự thảo kế hoạch 5 năm Tổng cục Tiêu chuẩn Đo lường Chất lượng thực hiện các nhiệm...</t>
-        </is>
-      </c>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Pháp luật về xây dựng và áp dụng tiêu chuẩn quy định cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch 5 năm xây dựng TCVN?»; nhãn cũ khong_dat question_ambiguous: 'Cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch' không ghim được chỗ đổi (cổng thông tin công khai); điểm b cùng khoản giao Tổng cục lấy ý kiến, hoàn chỉnh dự thảo kế hoạch, và điểm c do Bộ trưởng phê duyệt, Bộ thông báo). Câu hỏi chốt việc công khai sau phê duyệt (điểm c), chạm chỗ đổi</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:bcce4ee0-2f37-11f1-927e-c7ac35ffa800:2024-11-14</t>
+          <t>vilextime:T4:provision:ada68200-2d45-11f1-95b6-e35525714d94:2024-11-22</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2725,37 +2653,37 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Thẩm quyền áp dụng biện pháp khắc phục hậu quả của Chủ tịch Ủy ban nhân dân cấp huyện trong lĩnh vực bổ trợ tư pháp được xác định ra sao?</t>
+          <t>Sau khi kế hoạch 5 năm xây dựng TCVN được phê duyệt, kế hoạch phải được công khai trên cổng thông tin điện tử của những cơ quan nào và trong thời hạn bao lâu?</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2024-11-14</t>
+          <t>2024-11-22</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2. Chủ tịch Ủy ban nhân dân cấp huyện có quyền:</t>
+          <t>2. Kế hoạch 5 năm xây dựng TCVN Nội dung kế hoạch 5 năm xây dựng TCVN bao gồm: lĩnh vực, đối tượng cụ thể cần xây dựng TCVN; loại tiêu chuẩn; số lượng TCVN cần xây dựng; thời gian thực hiện; nguồn kinh phí và kinh phí dự kiến. Lập, phê duyệt, điều chỉnh, bổ sung kế hoạch 5 năm xây dựng TCVN thực hiện theo trình tự sau đây:</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d) Áp dụng biện pháp khắc phục hậu quả quy định tại các điểm a, e và i khoản 1 Điều 28 Luật Xử lý vi phạm hành chính; các điểm a, b, đ, l, m và n khoản 3 Điều 3 Nghị định này.</t>
+          <t>c) Phê duyệt kế hoạch 5 năm Bộ trưởng Bộ Khoa học và Công nghệ tổ chức xem xét, phê duyệt kế hoạch 5 năm xây dựng TCVN. Bộ Khoa học và Công nghệ thông báo kế hoạch đã được phê duyệt đến các bộ, ngành, tổ chức liên quan và công khai trên Cổng thông tin điện tử của Bộ Khoa học và Công nghệ, Cổng thông tin điện tử của Ủy ban Tiêu chuẩn Đo lường Chất lượng Quốc gia trong thời hạn 30 (ba mươi) ngày, kể từ ngày kế hoạch được phê duyệt;</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Điểm d Khoản 2 Điều 83</t>
+          <t>Điểm c Khoản 2 Điều 4</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>82/2020/NĐ-CP</t>
+          <t>11/2021/TT-BKHCN</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=143024</t>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=152575</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2770,16 +2698,21 @@
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Pháp luật về xây dựng và áp dụng tiêu chuẩn quy định cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch 5 năm xây dựng TCVN?»; nhãn cũ khong_dat question_ambiguous: 'Cơ quan nào phối hợp trong việc xây dựng và thông báo kế hoạch' không ghim được chỗ đổi (cổng thông tin công khai); điểm b cùng khoản giao Tổng cục lấy ý kiến, hoàn chỉnh dự thảo kế hoạch, và điểm c do Bộ trưởng phê duyệt, Bộ thông báo). Câu hỏi chốt việc công khai sau phê duyệt (điểm c), chạm chỗ đổi</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:bdb196ac-df3f-11f0-a53b-49fbe419b389:2025-06-23</t>
+          <t>vilextime:T4:provision:bcce4ee0-2f37-11f1-927e-c7ac35ffa800:2024-11-14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2789,37 +2722,37 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Khi hoạt động của bãi cất, hạ cánh trên boong tàu vi phạm điều kiện, quyết định đóng bãi phải được thông báo cho những bộ nào?</t>
+          <t>Thẩm quyền áp dụng biện pháp khắc phục hậu quả của Chủ tịch Ủy ban nhân dân cấp huyện trong lĩnh vực bổ trợ tư pháp được xác định ra sao?</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2025-06-23</t>
+          <t>2024-11-14</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Điều 16. Trình tự, thủ tục đóng bãi cất, hạ cánh trên boong tàu</t>
+          <t>2. Chủ tịch Ủy ban nhân dân cấp huyện có quyền:</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3. Khi hoạt động của bãi cất, hạ cánh vi phạm một trong các điều kiện quy định tại điểm a, b, c, d, đ của khoản 2 Điều 10; Bộ Tổng Tham mưu ra quyết định đóng bãi cất, hạ cánh và thông báo với Bộ Xây dựng, chủ sở hữu tàu và các cơ quan, tổ chức, cá nhân liên quan.</t>
+          <t>d) Áp dụng biện pháp khắc phục hậu quả quy định tại các điểm a, e và i khoản 1 Điều 28 Luật Xử lý vi phạm hành chính; các điểm a, b, đ, l, m và n khoản 3 Điều 3 Nghị định này.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Khoản 3 Điều 16</t>
+          <t>Điểm d Khoản 2 Điều 83</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>42/2016/NĐ-CP</t>
+          <t>82/2020/NĐ-CP</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141668</t>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=143024</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2839,11 +2772,12 @@
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:dcf457d0-3b96-11f1-b174-b5c1cf7b0c30:2026-08-09</t>
+          <t>vilextime:T4:provision:bdb196ac-df3f-11f0-a53b-49fbe419b389:2025-06-23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2853,37 +2787,37 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Khi Ủy ban nhân dân cấp tỉnh thực hiện nhiệm vụ quản lý vận tải đường bộ, cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào?</t>
+          <t>Khi hoạt động của bãi cất, hạ cánh trên boong tàu vi phạm điều kiện, quyết định đóng bãi phải được thông báo cho những bộ nào?</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2025-06-23</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Điều 73. Ủy ban nhân dân cấp tỉnh</t>
+          <t>Điều 16. Trình tự, thủ tục đóng bãi cất, hạ cánh trên boong tàu</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2. Phối hợp với Ủy ban nhân dân cấp tỉnh có tuyến xe buýt đi qua để thống nhất thực hiện các nhiệm vụ nêu tại khoản 3 Điều 5 của Nghị định này. Thống nhất với Bộ Giao thông vận tải trước khi mở tuyến xe buýt có điểm đầu hoặc điểm cuối nằm trong khu vực cảng hàng không.</t>
+          <t>3. Khi hoạt động của bãi cất, hạ cánh vi phạm một trong các điều kiện quy định tại điểm a, b, c, d, đ của khoản 2 Điều 10; Bộ Tổng Tham mưu ra quyết định đóng bãi cất, hạ cánh và thông báo với Bộ Xây dựng, chủ sở hữu tàu và các cơ quan, tổ chức, cá nhân liên quan.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Khoản 2 Điều 73</t>
+          <t>Khoản 3 Điều 16</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>158/2024/NĐ-CP</t>
+          <t>42/2016/NĐ-CP</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=173412</t>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=141668</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2893,29 +2827,22 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>unanswerable_as_asked</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Câu hỏi hỏi 'cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào', nhưng khoản 2 không nói về sở; chỗ đổi là Bộ phải thống nhất trước khi mở tuyến xe buýt vào cảng hàng không (Bộ Giao thông vận tải → Bộ Xây dựng)</t>
-        </is>
-      </c>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:dcf457d0-3b96-11f1-b174-b5c1cf7b0c30:2026-08-10</t>
+          <t>vilextime:T4:provision:dcf457d0-3b96-11f1-b174-b5c1cf7b0c30:2026-08-09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2925,12 +2852,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Khi Ủy ban nhân dân cấp tỉnh thực hiện nhiệm vụ quản lý vận tải đường bộ, cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào?</t>
+          <t>Trước khi mở tuyến xe buýt đi đến hoặc xuất phát từ khu vực cảng hàng không, Ủy ban nhân dân cấp tỉnh phải thống nhất với bộ nào?</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2940,7 +2867,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2. Phối hợp với Ủy ban nhân dân cấp tỉnh có tuyến xe buýt đi qua để thống nhất thực hiện các nhiệm vụ nêu tại khoản 3 Điều 5 của Nghị định này. Thống nhất với Bộ Xây dựng trước khi mở tuyến xe buýt có điểm đầu hoặc điểm cuối nằm trong khu vực cảng hàng không.</t>
+          <t>2. Phối hợp với Ủy ban nhân dân cấp tỉnh có tuyến xe buýt đi qua để thống nhất thực hiện các nhiệm vụ nêu tại khoản 3 Điều 5 của Nghị định này. Thống nhất với Bộ Giao thông vận tải trước khi mở tuyến xe buýt có điểm đầu hoặc điểm cuối nằm trong khu vực cảng hàng không.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2965,29 +2892,26 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>unanswerable_as_asked</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Câu hỏi hỏi 'cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào', nhưng khoản 2 không nói về sở; chỗ đổi là Bộ phải thống nhất trước khi mở tuyến xe buýt vào cảng hàng không (Bộ Giao thông vận tải → Bộ Xây dựng)</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi Ủy ban nhân dân cấp tỉnh thực hiện nhiệm vụ quản lý vận tải đường bộ, cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào?»; nhãn cũ khong_dat unanswerable_as_asked: Câu hỏi hỏi 'cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào', nhưng khoản 2 không nói về sở; chỗ đổi là Bộ phải thống nhất trước khi mở tuyến xe buýt vào cảng hàng không (Bộ Giao thông vận tải → Bộ Xây dựng)). Câu hỏi hỏi bộ phải thống nhất, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:fc79fb04-2c7e-11f1-9a1a-67adfcf2b37c:2024-11-21</t>
+          <t>vilextime:T4:provision:dcf457d0-3b96-11f1-b174-b5c1cf7b0c30:2026-08-10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2997,37 +2921,37 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Một tổ chức nhận văn bản thông báo kết quả đánh giá hồ sơ tuyển chọn nhiệm vụ của chương trình năng suất chất lượng thì văn bản đó do cơ quan nào ban hành?</t>
+          <t>Trước khi mở tuyến xe buýt đi đến hoặc xuất phát từ khu vực cảng hàng không, Ủy ban nhân dân cấp tỉnh phải thống nhất với bộ nào?</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2024-11-21</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Điều 19. Chuyên gia tư vấn độc lập đánh giá hồ sơ đăng ký tuyển chọn, giao trực tiếp thực hiện nhiệm vụ Việc đánh giá của chuyên gia tư vấn độc lập đối với hồ sơ đăng ký tuyển chọn, giao trực tiếp thực hiện nhiệm vụ được thực hiện theo quy định tại Điều 18, 19, 20 Chương IV Thông tư số 08/2017/TT-BKHCN. Áp dụng cụ thể đối với các nhiệm vụ thuộc Chương trình như sau:</t>
+          <t>Điều 73. Ủy ban nhân dân cấp tỉnh</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>6. Trong thời hạn 10 ngày kể từ ngày nhận được văn bản thông báo của tổng cục Tiêu chuẩn Đo lường Chất lượng theo quy định tại khoản 5 Điều này, tổ chức được kiến nghị chủ trì thực hiện nhiệm vụ hoàn thiện và gửi hồ sơ cho Tổng cục Tiêu chuẩn Đo lường Chất lượng.</t>
+          <t>2. Phối hợp với Ủy ban nhân dân cấp tỉnh có tuyến xe buýt đi qua để thống nhất thực hiện các nhiệm vụ nêu tại khoản 3 Điều 5 của Nghị định này. Thống nhất với Bộ Xây dựng trước khi mở tuyến xe buýt có điểm đầu hoặc điểm cuối nằm trong khu vực cảng hàng không.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Khoản 6 Điều 19</t>
+          <t>Khoản 2 Điều 73</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>15/2022/TT-BKHCN</t>
+          <t>158/2024/NĐ-CP</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160095</t>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=173412</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3037,29 +2961,26 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Văn bản thông báo vẫn là của 'tổng cục Tiêu chuẩn Đo lường Chất lượng' ở cả hai mốc (chữ viết thường nên lần thay tên không chạm tới); chỗ đổi là nơi nhận hồ sơ (Tổng cục → Ủy ban), câu hỏi không hỏi</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Khi Ủy ban nhân dân cấp tỉnh thực hiện nhiệm vụ quản lý vận tải đường bộ, cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào?»; nhãn cũ khong_dat unanswerable_as_asked: Câu hỏi hỏi 'cơ quan chuyên môn về giao thông ở địa phương được gọi tên theo sở nào', nhưng khoản 2 không nói về sở; chỗ đổi là Bộ phải thống nhất trước khi mở tuyến xe buýt vào cảng hàng không (Bộ Giao thông vận tải → Bộ Xây dựng)). Câu hỏi hỏi bộ phải thống nhất, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>vilextime:T4:provision:fc79fb04-2c7e-11f1-9a1a-67adfcf2b37c:2024-11-22</t>
+          <t>vilextime:T4:provision:fc79fb04-2c7e-11f1-9a1a-67adfcf2b37c:2024-11-21</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3069,12 +2990,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Một tổ chức nhận văn bản thông báo kết quả đánh giá hồ sơ tuyển chọn nhiệm vụ của chương trình năng suất chất lượng thì văn bản đó do cơ quan nào ban hành?</t>
+          <t>Sau khi nhận văn bản thông báo kết quả đánh giá hồ sơ tuyển chọn nhiệm vụ của chương trình năng suất chất lượng, tổ chức được kiến nghị chủ trì phải hoàn thiện và gửi hồ sơ cho cơ quan nào trong thời hạn bao lâu?</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2024-11-22</t>
+          <t>2024-11-21</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3084,7 +3005,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>6. Trong thời hạn 10 ngày kể từ ngày nhận được văn bản thông báo của tổng cục Tiêu chuẩn Đo lường Chất lượng theo quy định tại khoản 5 Điều này, tổ chức được kiến nghị chủ trì thực hiện nhiệm vụ hoàn thiện và gửi hồ sơ cho Ủy ban Tiêu chuẩn Đo lường Chất lượng Quốc gia.</t>
+          <t>6. Trong thời hạn 10 ngày kể từ ngày nhận được văn bản thông báo của tổng cục Tiêu chuẩn Đo lường Chất lượng theo quy định tại khoản 5 Điều này, tổ chức được kiến nghị chủ trì thực hiện nhiệm vụ hoàn thiện và gửi hồ sơ cho Tổng cục Tiêu chuẩn Đo lường Chất lượng.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3109,24 +3030,90 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>khong_dat</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>group_mismatch</t>
-        </is>
-      </c>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Văn bản thông báo vẫn là của 'tổng cục Tiêu chuẩn Đo lường Chất lượng' ở cả hai mốc (chữ viết thường nên lần thay tên không chạm tới); chỗ đổi là nơi nhận hồ sơ (Tổng cục → Ủy ban), câu hỏi không hỏi</t>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Một tổ chức nhận văn bản thông báo kết quả đánh giá hồ sơ tuyển chọn nhiệm vụ của chương trình năng suất chất lượng thì văn bản đó do cơ quan nào ban hành?»; nhãn cũ khong_dat group_mismatch: Văn bản thông báo vẫn là của 'tổng cục Tiêu chuẩn Đo lường Chất lượng' ở cả hai mốc (chữ viết thường nên lần thay tên không chạm tới); chỗ đổi là nơi nhận hồ sơ (Tổng cục → Ủy ban), câu hỏi không hỏi). Câu hỏi hỏi nơi nhận hồ sơ, chạm chỗ đổi</t>
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>vilextime:T4:provision:fc79fb04-2c7e-11f1-9a1a-67adfcf2b37c:2024-11-22</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Sau khi nhận văn bản thông báo kết quả đánh giá hồ sơ tuyển chọn nhiệm vụ của chương trình năng suất chất lượng, tổ chức được kiến nghị chủ trì phải hoàn thiện và gửi hồ sơ cho cơ quan nào trong thời hạn bao lâu?</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2024-11-22</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Điều 19. Chuyên gia tư vấn độc lập đánh giá hồ sơ đăng ký tuyển chọn, giao trực tiếp thực hiện nhiệm vụ Việc đánh giá của chuyên gia tư vấn độc lập đối với hồ sơ đăng ký tuyển chọn, giao trực tiếp thực hiện nhiệm vụ được thực hiện theo quy định tại Điều 18, 19, 20 Chương IV Thông tư số 08/2017/TT-BKHCN. Áp dụng cụ thể đối với các nhiệm vụ thuộc Chương trình như sau:</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>6. Trong thời hạn 10 ngày kể từ ngày nhận được văn bản thông báo của tổng cục Tiêu chuẩn Đo lường Chất lượng theo quy định tại khoản 5 Điều này, tổ chức được kiến nghị chủ trì thực hiện nhiệm vụ hoàn thiện và gửi hồ sơ cho Ủy ban Tiêu chuẩn Đo lường Chất lượng Quốc gia.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Khoản 6 Điều 19</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>15/2022/TT-BKHCN</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=160095</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>claude-opus-5-5</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Chấm lại 28/09 trên câu hỏi viết lại (câu cũ: «Một tổ chức nhận văn bản thông báo kết quả đánh giá hồ sơ tuyển chọn nhiệm vụ của chương trình năng suất chất lượng thì văn bản đó do cơ quan nào ban hành?»; nhãn cũ khong_dat group_mismatch: Văn bản thông báo vẫn là của 'tổng cục Tiêu chuẩn Đo lường Chất lượng' ở cả hai mốc (chữ viết thường nên lần thay tên không chạm tới); chỗ đổi là nơi nhận hồ sơ (Tổng cục → Ủy ban), câu hỏi không hỏi). Câu hỏi hỏi nơi nhận hồ sơ, chạm chỗ đổi</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>